<commit_message>
files saved to a folder in C and separate executable for handling lost files
</commit_message>
<xml_diff>
--- a/Buick_failed_to_download.xlsx
+++ b/Buick_failed_to_download.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nir\PycharmProjects\AdExtracterBot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAF9BA44-7DE1-4B8B-9CB4-474DE71FF02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30D65B62-3BF7-4809-BB2C-8A5C09D2705E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,21 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
     <t>Values</t>
-  </si>
-  <si>
-    <t>15255489341</t>
-  </si>
-  <si>
-    <t>15285837211</t>
-  </si>
-  <si>
-    <t>586341564</t>
-  </si>
-  <si>
-    <t>15282641480</t>
   </si>
 </sst>
 </file>
@@ -90,11 +78,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -409,23 +398,23 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
+      <c r="A2" s="2">
+        <v>15255489341</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
+      <c r="A3" s="2">
+        <v>15285837211</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
+      <c r="A4" s="2">
+        <v>586341564</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
+      <c r="A5" s="2">
+        <v>15282641480</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>